<commit_message>
EPBDS-6960 Allow this and current to access containing spreadsheet cells
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/3-Calculations/Spreadsheets.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/3-Calculations/Spreadsheets.xlsx
@@ -1733,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:R46"/>
+  <dimension ref="B2:X126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2065,38 +2065,94 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>= $Vehicles[1].$Premium</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Method String PremiumSummary(SpreadsheetResultVehiclePremium result)</t>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MatchWithThis</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>= $Vehicles[select first having $Premium == this.$Premium].$Premium</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>return "Base " + result.$Base + ", premium " + result.$Premium;</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>A step can declare the type of a nested result, "First : SpreadsheetResultVehiclePremium", to read its cells later. "$Value$Premium($Vehicles)" names the column as well as the row. A cell of a call is read right away, "VehiclePremium(vehicle).$Premium", and "getFieldValue("$Value$Premium")" reads a cell by its full name given as text. A result kept as Object is cast back with "(SpreadsheetResult[]) value".</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16.5" customHeight="1">
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>A test checks the cells of nested results: "_res_.$Value$Vehicles[1].$Value$Premium" reads the premium of the second vehicle.</t>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MatchWithCurrent</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>= $Vehicles[select first having $Premium == current.$Premium].$Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MatchWithFullThis</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>= $Vehicles[select first having $Premium == this.$Value$Premium].$Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>MatchWithFullCurrent</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>= $Vehicles[select first having $Premium == current.$Value$Premium].$Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MatchWithNamedVehicle</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>= $Vehicles[(vehicle) select first having vehicle.$Premium == current.$Premium].$Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FirstByElementPremium</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>= $Vehicles[select first having $Premium == 400].$Premium</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Test PolicyPremium PolicyPremiumTest</t>
+          <t>Method String PremiumSummary(SpreadsheetResultVehiclePremium result)</t>
         </is>
       </c>
       <c r="C43" s="4" t="n"/>
@@ -2105,261 +2161,1171 @@
       <c r="F43" s="4" t="n"/>
       <c r="G43" s="4" t="n"/>
       <c r="H43" s="4" t="n"/>
-      <c r="I43" s="4" t="n"/>
-      <c r="J43" s="4" t="n"/>
-      <c r="K43" s="4" t="n"/>
-      <c r="L43" s="4" t="n"/>
-      <c r="M43" s="4" t="n"/>
-      <c r="N43" s="4" t="n"/>
-      <c r="O43" s="4" t="n"/>
-      <c r="P43" s="4" t="n"/>
-      <c r="Q43" s="4" t="n"/>
-      <c r="R43" s="5" t="n"/>
+      <c r="I43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>return "Base " + result.$Base + ", premium " + result.$Premium;</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>A step can declare the type of a nested result, "First : SpreadsheetResultVehiclePremium", to read its cells later. "$Value$Premium($Vehicles)" names the column as well as the row. A cell of a call is read right away, "VehiclePremium(vehicle).$Premium", and "getFieldValue("$Value$Premium")" reads a cell by its full name given as text. A result kept as Object is cast back with "(SpreadsheetResult[]) value". When a SELECT condition uses a spreadsheet cell that also exists in an array element, qualify the cell of the containing spreadsheet with this or current: this.$Premium and current.$Premium.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>A test checks the cells of nested results: "_res_.$Value$Vehicles[1].$Value$Premium" reads the premium of the second vehicle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Test PolicyPremium PolicyPremiumTest</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
+      <c r="J50" s="4" t="n"/>
+      <c r="K50" s="4" t="n"/>
+      <c r="L50" s="4" t="n"/>
+      <c r="M50" s="4" t="n"/>
+      <c r="N50" s="4" t="n"/>
+      <c r="O50" s="4" t="n"/>
+      <c r="P50" s="4" t="n"/>
+      <c r="Q50" s="4" t="n"/>
+      <c r="R50" s="5" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>vehicles[0].id</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C51" s="9" t="inlineStr">
         <is>
           <t>vehicles[0].value</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D51" s="9" t="inlineStr">
         <is>
           <t>vehicles[0].age</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr">
         <is>
           <t>vehicles[1].id</t>
         </is>
       </c>
-      <c r="F44" s="9" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>vehicles[1].value</t>
         </is>
       </c>
-      <c r="G44" s="9" t="inlineStr">
+      <c r="G51" s="9" t="inlineStr">
         <is>
           <t>vehicles[1].age</t>
         </is>
       </c>
-      <c r="H44" s="9" t="inlineStr">
+      <c r="H51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Value$Total</t>
         </is>
       </c>
-      <c r="I44" s="9" t="inlineStr">
+      <c r="I51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Value$Highest</t>
         </is>
       </c>
-      <c r="J44" s="9" t="inlineStr">
+      <c r="J51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Value$OldCars</t>
         </is>
       </c>
-      <c r="K44" s="9" t="inlineStr">
+      <c r="K51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Value$Vehicles[1].$Value$Premium</t>
         </is>
       </c>
-      <c r="L44" s="9" t="inlineStr">
+      <c r="L51" s="9" t="inlineStr">
         <is>
           <t>_res_.$Value$Summary</t>
         </is>
       </c>
-      <c r="M44" s="9" t="inlineStr">
+      <c r="M51" s="9" t="inlineStr">
         <is>
           <t>_res_.$FirstBase</t>
         </is>
       </c>
-      <c r="N44" s="9" t="inlineStr">
+      <c r="N51" s="9" t="inlineStr">
         <is>
           <t>_res_.$AllPremiums</t>
         </is>
       </c>
-      <c r="O44" s="9" t="inlineStr">
+      <c r="O51" s="9" t="inlineStr">
         <is>
           <t>_res_.$DirectCell</t>
         </is>
       </c>
-      <c r="P44" s="9" t="inlineStr">
+      <c r="P51" s="9" t="inlineStr">
         <is>
           <t>_res_.$CellByName</t>
         </is>
       </c>
-      <c r="Q44" s="9" t="inlineStr">
+      <c r="Q51" s="9" t="inlineStr">
         <is>
           <t>_res_.$FirstPremium</t>
         </is>
       </c>
-      <c r="R44" s="9" t="inlineStr">
+      <c r="R51" s="9" t="inlineStr">
         <is>
           <t>_res_.$BackToResults[1].$Value$Premium</t>
         </is>
       </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="6" t="inlineStr">
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>_res_.$MatchWithThis</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>_res_.$MatchWithCurrent</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>_res_.$MatchWithFullThis</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>_res_.$MatchWithFullCurrent</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>_res_.$MatchWithNamedVehicle</t>
+        </is>
+      </c>
+      <c r="X51" t="inlineStr">
+        <is>
+          <t>_res_.$FirstByElementPremium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>Vehicle 1</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Value 1</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>Age 1</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>Vehicle 2</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Value 2</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>Age 2</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
+      <c r="I52" s="6" t="inlineStr">
         <is>
           <t>Highest</t>
         </is>
       </c>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="J52" s="6" t="inlineStr">
         <is>
           <t>Old Cars</t>
         </is>
       </c>
-      <c r="K45" s="6" t="inlineStr">
+      <c r="K52" s="6" t="inlineStr">
         <is>
           <t>Second Premium</t>
         </is>
       </c>
-      <c r="L45" s="6" t="inlineStr">
+      <c r="L52" s="6" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="M45" s="6" t="inlineStr">
+      <c r="M52" s="6" t="inlineStr">
         <is>
           <t>First Base</t>
         </is>
       </c>
-      <c r="N45" s="6" t="inlineStr">
+      <c r="N52" s="6" t="inlineStr">
         <is>
           <t>All Premiums</t>
         </is>
       </c>
-      <c r="O45" s="6" t="inlineStr">
+      <c r="O52" s="6" t="inlineStr">
         <is>
           <t>Direct Cell</t>
         </is>
       </c>
-      <c r="P45" s="6" t="inlineStr">
+      <c r="P52" s="6" t="inlineStr">
         <is>
           <t>Cell By Name</t>
         </is>
       </c>
-      <c r="Q45" s="6" t="inlineStr">
+      <c r="Q52" s="6" t="inlineStr">
         <is>
           <t>First Premium</t>
         </is>
       </c>
-      <c r="R45" s="6" t="inlineStr">
+      <c r="R52" s="6" t="inlineStr">
         <is>
           <t>Cast Back</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="7" t="inlineStr">
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Match With This</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Match With Current</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Full This</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Full Current</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>Named Vehicle</t>
+        </is>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>Element Premium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="7" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="C46" s="7" t="n">
+      <c r="C53" s="7" t="n">
         <v>20000</v>
       </c>
-      <c r="D46" s="7" t="n">
+      <c r="D53" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="7" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="F46" s="7" t="n">
+      <c r="F53" s="7" t="n">
         <v>8000</v>
       </c>
-      <c r="G46" s="7" t="n">
+      <c r="G53" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="H46" s="10" t="n">
+      <c r="H53" s="10" t="n">
         <v>592</v>
       </c>
-      <c r="I46" s="10" t="n">
+      <c r="I53" s="10" t="n">
         <v>400</v>
       </c>
-      <c r="J46" s="10" t="n">
+      <c r="J53" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="K46" s="10" t="n">
+      <c r="K53" s="10" t="n">
         <v>192</v>
       </c>
-      <c r="L46" s="10" t="inlineStr">
+      <c r="L53" s="10" t="inlineStr">
         <is>
           <t>Base 400.0, premium 400.0</t>
         </is>
       </c>
-      <c r="M46" s="10" t="n">
+      <c r="M53" s="10" t="n">
         <v>400</v>
       </c>
-      <c r="N46" s="10" t="inlineStr">
+      <c r="N53" s="10" t="inlineStr">
         <is>
           <t>400, 192</t>
         </is>
       </c>
-      <c r="O46" s="10" t="n">
+      <c r="O53" s="10" t="n">
         <v>192</v>
       </c>
-      <c r="P46" s="10" t="n">
+      <c r="P53" s="10" t="n">
         <v>192</v>
       </c>
-      <c r="Q46" s="10" t="n">
+      <c r="Q53" s="10" t="n">
         <v>400</v>
       </c>
-      <c r="R46" s="10" t="n">
+      <c r="R53" s="10" t="n">
         <v>192</v>
       </c>
+      <c r="S53" t="n">
+        <v>192</v>
+      </c>
+      <c r="T53" t="n">
+        <v>192</v>
+      </c>
+      <c r="U53" t="n">
+        <v>192</v>
+      </c>
+      <c r="V53" t="n">
+        <v>192</v>
+      </c>
+      <c r="W53" t="n">
+        <v>192</v>
+      </c>
+      <c r="X53" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>When SELECT reads an array of spreadsheet results, an unqualified cell belongs to each result. this or current reads a cell of the spreadsheet containing the formula. A named element also makes the comparison explicit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult SelectionItem(Integer key)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>= key</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>A condition can use more than one cell of the containing spreadsheet. The selected claim must have the required type and a year within the allowed period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult ClaimYear(Integer type, Integer years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>= type</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>NumberOfYears</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>= years</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult PolicyClaims(Integer[] types, Integer[] years, Integer liabType, Integer[] allowedYears)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>LiabType</t>
+        </is>
+      </c>
+      <c r="C70" s="8" t="inlineStr">
+        <is>
+          <t>= liabType</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>= allowedYears</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Claims</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>= ClaimYear(types, years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>MatchingYears</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>= $Claims[select first having $Type == current.$LiabType &amp;&amp; $NumberOfYears &lt; length(current.$Years)].$NumberOfYears</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Test PolicyClaims PolicyClaimsTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>types</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>liabType</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>allowedYears</t>
+        </is>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$MatchingYears</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Claim Types</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Required Type</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>Allowed Years</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>Selected Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>2, 2</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>4, 1</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>0, 0, 0</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>A one-row spreadsheet can name another column with this.$OtherColumn or current.$OtherColumn. In a spreadsheet with several columns, both use the column of their own formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult OneRowSelection(Integer[] keys, Integer desired)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Desired</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>OtherColumn</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>FromThis</t>
+        </is>
+      </c>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>FromCurrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>= desired</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>= SelectionItem(keys)</t>
+        </is>
+      </c>
+      <c r="E84" s="8" t="inlineStr">
+        <is>
+          <t>= desired</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>= $Items[select first having $Key == this.$OtherColumn].$Key</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>= $Items[select first having $Key == current.$OtherColumn].$Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Test OneRowSelection OneRowSelectionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="9" t="inlineStr">
+        <is>
+          <t>keys</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>desired</t>
+        </is>
+      </c>
+      <c r="D87" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$OtherColumn$Value</t>
+        </is>
+      </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromThis$Value</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromCurrent$Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>Keys</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>Desired</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>Other Column</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>This</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E89" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult TwoColumnSelection()</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>First</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Wanted</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>= 2</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>= 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>FromThis</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>= this.$Wanted</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>= this.$Wanted</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>FromCurrent</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>= current.$Wanted</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>= current.$Wanted</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Test TwoColumnSelection TwoColumnSelectionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$First$FromThis</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$First$FromCurrent</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Second$FromThis</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Second$FromCurrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>First This</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>First Current</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>Second This</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Second Current</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E100" s="7" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>A parameter named current keeps its parameter value. Use this to read a spreadsheet cell with the same purpose inside SELECT. When no parameter has that name, current can read a spreadsheet cell in any formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult ParameterCurrent(Integer current, Integer[] keys)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C105" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="B106" s="7" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="C106" s="8" t="inlineStr">
+        <is>
+          <t>= current + 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>= SelectionItem(keys)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="7" t="inlineStr">
+        <is>
+          <t>CurrentValue</t>
+        </is>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>= current</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>FromParameter</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>= $Items[select first having $Key == current].$Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="7" t="inlineStr">
+        <is>
+          <t>FromSpreadsheet</t>
+        </is>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>= $Items[select first having $Key == this.$Key].$Key</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Test ParameterCurrent ParameterCurrentTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>keys</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$CurrentValue</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromParameter</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FromSpreadsheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>Current Parameter</t>
+        </is>
+      </c>
+      <c r="C114" s="6" t="inlineStr">
+        <is>
+          <t>Keys</t>
+        </is>
+      </c>
+      <c r="D114" s="6" t="inlineStr">
+        <is>
+          <t>Parameter Value</t>
+        </is>
+      </c>
+      <c r="E114" s="6" t="inlineStr">
+        <is>
+          <t>Selected By Parameter</t>
+        </is>
+      </c>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>Selected By Spreadsheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t>2, 3</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E115" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F115" s="7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t>7, 8</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E116" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="F116" s="7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult CurrentCell()</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C119" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>= 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>= current.$A + 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Test CurrentCell CurrentCellTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="7" t="n">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="12">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B39:I39"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B43:R43"/>
-    <mergeCell ref="B41:I41"/>
+    <mergeCell ref="B61:R61"/>
+    <mergeCell ref="B55:R55"/>
+    <mergeCell ref="B47:R47"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B80:R80"/>
     <mergeCell ref="B4:I4"/>
+    <mergeCell ref="B102:R102"/>
     <mergeCell ref="B17:I17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>